<commit_message>
Add TOTAL sentinel for population-level constraints
Introduce TOTAL sentinel to allow constraints that span the whole population rather than a single decision. Validator now accepts TOTAL, constraint linearisation and summation iterate over all decisions when TOTAL is used, and KPI evaluation was refactored to operate on (leaf,decision) pairs and to produce per-decision and TOTAL realised values. UI updated to expose TOTAL in decision dropdowns. Added an example problem using TOTAL (credit_fixed_accept_min_bad.json) and updated/renamed notebooks, model path (titanic_tree.pkl -> notebooks/models/), and solution files accordingly.
</commit_message>
<xml_diff>
--- a/notebooks/solutions/credit_solution.xlsx
+++ b/notebooks/solutions/credit_solution.xlsx
@@ -3879,7 +3879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3959,16 +3959,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kAcceptedRatio</t>
+          <t>kBadRatio</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Accept</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.2212</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
@@ -3982,15 +3982,51 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Reject</t>
+          <t>Accept</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>kAcceptedRatio</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>kAcceptedRatio</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.4116</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>